<commit_message>
Nuevo módulo AF y cambios en carga masiva traslado y uso cajas
</commit_message>
<xml_diff>
--- a/public/template_carga_cajas.xlsx
+++ b/public/template_carga_cajas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asistemas01uio\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C36F01-4220-4336-BDB9-0BE4E70F6DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{68188C41-D8CB-47AE-B640-790163AE699B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{CFB3BBA5-7F5E-4E9D-B5B3-D05F4D8BAEA6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{CFB3BBA5-7F5E-4E9D-B5B3-D05F4D8BAEA6}"/>
   </bookViews>
   <sheets>
     <sheet name="Encabezado" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>CodigoCaja</t>
   </si>
@@ -51,12 +51,6 @@
     <t>ClaseCaja</t>
   </si>
   <si>
-    <t>TRIMANO.GYE.0009</t>
-  </si>
-  <si>
-    <t>AR-1740</t>
-  </si>
-  <si>
     <t>CodigoItem</t>
   </si>
   <si>
@@ -67,12 +61,6 @@
   </si>
   <si>
     <t>LoteItem</t>
-  </si>
-  <si>
-    <t>AF</t>
-  </si>
-  <si>
-    <t>AR-1741-2024</t>
   </si>
   <si>
     <t>Descripcion</t>
@@ -481,19 +469,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
       <c r="B2" s="3">
-        <v>45819</v>
-      </c>
-      <c r="C2" s="2">
-        <v>2010</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
+        <f ca="1">TODAY()</f>
+        <v>45839</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -510,40 +493,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
-      </c>
     </row>
-    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2">
-        <v>980394998</v>
-      </c>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>

</xml_diff>